<commit_message>
Fehlerhafte Excel-Datei hochgeladen (Test)
</commit_message>
<xml_diff>
--- a/daten/projekte.xlsx
+++ b/daten/projekte.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -661,9 +661,6 @@
       <c r="D8" t="n">
         <v>100</v>
       </c>
-      <c r="E8" t="n">
-        <v>95</v>
-      </c>
       <c r="F8" s="3" t="n">
         <v>46280</v>
       </c>
@@ -717,6 +714,32 @@
         <v>0</v>
       </c>
       <c r="F10" s="3" t="n">
+        <v>46280</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Schichtplanung</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Produktion</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>laufend</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>150</v>
+      </c>
+      <c r="E11" t="n">
+        <v>160</v>
+      </c>
+      <c r="F11" s="3" t="n">
         <v>46280</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Startstand wiederhergestellt (Datenstand 01.09.2026)
</commit_message>
<xml_diff>
--- a/daten/projekte.xlsx
+++ b/daten/projekte.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -506,10 +506,10 @@
         <v>120</v>
       </c>
       <c r="E2" t="n">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>46280</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="3">
@@ -532,10 +532,10 @@
         <v>80</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>46280</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="4">
@@ -561,7 +561,7 @@
         <v>60</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>46280</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="5">
@@ -584,10 +584,10 @@
         <v>150</v>
       </c>
       <c r="E5" t="n">
-        <v>155</v>
+        <v>140</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>46280</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="6">
@@ -603,17 +603,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>laufend</t>
+          <t>geplant</t>
         </is>
       </c>
       <c r="D6" t="n">
         <v>40</v>
       </c>
       <c r="E6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>46280</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="7">
@@ -639,7 +639,7 @@
         <v>55</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>46280</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="8">
@@ -661,8 +661,11 @@
       <c r="D8" t="n">
         <v>100</v>
       </c>
+      <c r="E8" t="n">
+        <v>90</v>
+      </c>
       <c r="F8" s="3" t="n">
-        <v>46280</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="9">
@@ -688,59 +691,7 @@
         <v>70</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>46280</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Datenschutzschulung</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Personal</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>geplant</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>30</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="3" t="n">
-        <v>46280</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Schichtplanung</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Produktion</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>laufend</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>150</v>
-      </c>
-      <c r="E11" t="n">
-        <v>160</v>
-      </c>
-      <c r="F11" s="3" t="n">
-        <v>46280</v>
+        <v>46266</v>
       </c>
     </row>
   </sheetData>

</xml_diff>